<commit_message>
feat: Connect live registration, profiles, and SOS alerts to Supabase cloud database
</commit_message>
<xml_diff>
--- a/Appium_Test_Report_300.xlsx
+++ b/Appium_Test_Report_300.xlsx
@@ -574,7 +574,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Execution Date: 2026-08-27 10:47:02</t>
+          <t>Execution Date: 2026-08-27 11:54:37</t>
         </is>
       </c>
     </row>
@@ -764,7 +764,7 @@
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>~11.30 seconds</t>
+          <t>~11.29 seconds</t>
         </is>
       </c>
       <c r="C15" s="10" t="inlineStr">
@@ -1201,7 +1201,7 @@
         </is>
       </c>
       <c r="K2" s="7" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="L2" s="7" t="inlineStr">
         <is>
@@ -1264,7 +1264,7 @@
         </is>
       </c>
       <c r="K3" s="10" t="n">
-        <v>17</v>
+        <v>44</v>
       </c>
       <c r="L3" s="10" t="inlineStr">
         <is>
@@ -1327,7 +1327,7 @@
         </is>
       </c>
       <c r="K4" s="7" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="L4" s="7" t="inlineStr">
         <is>
@@ -1390,7 +1390,7 @@
         </is>
       </c>
       <c r="K5" s="10" t="n">
-        <v>48</v>
+        <v>58</v>
       </c>
       <c r="L5" s="10" t="inlineStr">
         <is>
@@ -1453,7 +1453,7 @@
         </is>
       </c>
       <c r="K6" s="7" t="n">
-        <v>25</v>
+        <v>56</v>
       </c>
       <c r="L6" s="7" t="inlineStr">
         <is>
@@ -1516,7 +1516,7 @@
         </is>
       </c>
       <c r="K7" s="10" t="n">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="L7" s="10" t="inlineStr">
         <is>
@@ -1579,7 +1579,7 @@
         </is>
       </c>
       <c r="K8" s="7" t="n">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="L8" s="7" t="inlineStr">
         <is>
@@ -1642,7 +1642,7 @@
         </is>
       </c>
       <c r="K9" s="10" t="n">
-        <v>58</v>
+        <v>20</v>
       </c>
       <c r="L9" s="10" t="inlineStr">
         <is>
@@ -1705,7 +1705,7 @@
         </is>
       </c>
       <c r="K10" s="7" t="n">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="L10" s="7" t="inlineStr">
         <is>
@@ -1768,7 +1768,7 @@
         </is>
       </c>
       <c r="K11" s="10" t="n">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="L11" s="10" t="inlineStr">
         <is>
@@ -1831,7 +1831,7 @@
         </is>
       </c>
       <c r="K12" s="7" t="n">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="L12" s="7" t="inlineStr">
         <is>
@@ -1894,7 +1894,7 @@
         </is>
       </c>
       <c r="K13" s="10" t="n">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="L13" s="10" t="inlineStr">
         <is>
@@ -1957,7 +1957,7 @@
         </is>
       </c>
       <c r="K14" s="7" t="n">
-        <v>58</v>
+        <v>19</v>
       </c>
       <c r="L14" s="7" t="inlineStr">
         <is>
@@ -2020,7 +2020,7 @@
         </is>
       </c>
       <c r="K15" s="10" t="n">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="L15" s="10" t="inlineStr">
         <is>
@@ -2083,7 +2083,7 @@
         </is>
       </c>
       <c r="K16" s="7" t="n">
-        <v>53</v>
+        <v>31</v>
       </c>
       <c r="L16" s="7" t="inlineStr">
         <is>
@@ -2146,7 +2146,7 @@
         </is>
       </c>
       <c r="K17" s="10" t="n">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="L17" s="10" t="inlineStr">
         <is>
@@ -2209,7 +2209,7 @@
         </is>
       </c>
       <c r="K18" s="7" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="L18" s="7" t="inlineStr">
         <is>
@@ -2272,7 +2272,7 @@
         </is>
       </c>
       <c r="K19" s="10" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="L19" s="10" t="inlineStr">
         <is>
@@ -2335,7 +2335,7 @@
         </is>
       </c>
       <c r="K20" s="7" t="n">
-        <v>50</v>
+        <v>23</v>
       </c>
       <c r="L20" s="7" t="inlineStr">
         <is>
@@ -2398,7 +2398,7 @@
         </is>
       </c>
       <c r="K21" s="10" t="n">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="L21" s="10" t="inlineStr">
         <is>
@@ -2461,7 +2461,7 @@
         </is>
       </c>
       <c r="K22" s="7" t="n">
-        <v>16</v>
+        <v>57</v>
       </c>
       <c r="L22" s="7" t="inlineStr">
         <is>
@@ -2524,7 +2524,7 @@
         </is>
       </c>
       <c r="K23" s="10" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="L23" s="10" t="inlineStr">
         <is>
@@ -2587,7 +2587,7 @@
         </is>
       </c>
       <c r="K24" s="7" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="L24" s="7" t="inlineStr">
         <is>
@@ -2650,7 +2650,7 @@
         </is>
       </c>
       <c r="K25" s="10" t="n">
-        <v>39</v>
+        <v>18</v>
       </c>
       <c r="L25" s="10" t="inlineStr">
         <is>
@@ -2713,7 +2713,7 @@
         </is>
       </c>
       <c r="K26" s="7" t="n">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="L26" s="7" t="inlineStr">
         <is>
@@ -2776,7 +2776,7 @@
         </is>
       </c>
       <c r="K27" s="10" t="n">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="L27" s="10" t="inlineStr">
         <is>
@@ -2839,7 +2839,7 @@
         </is>
       </c>
       <c r="K28" s="7" t="n">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="L28" s="7" t="inlineStr">
         <is>
@@ -2902,7 +2902,7 @@
         </is>
       </c>
       <c r="K29" s="10" t="n">
-        <v>31</v>
+        <v>52</v>
       </c>
       <c r="L29" s="10" t="inlineStr">
         <is>
@@ -2965,7 +2965,7 @@
         </is>
       </c>
       <c r="K30" s="7" t="n">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="L30" s="7" t="inlineStr">
         <is>
@@ -3028,7 +3028,7 @@
         </is>
       </c>
       <c r="K31" s="10" t="n">
-        <v>24</v>
+        <v>58</v>
       </c>
       <c r="L31" s="10" t="inlineStr">
         <is>
@@ -3091,7 +3091,7 @@
         </is>
       </c>
       <c r="K32" s="7" t="n">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="L32" s="7" t="inlineStr">
         <is>
@@ -3154,7 +3154,7 @@
         </is>
       </c>
       <c r="K33" s="10" t="n">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="L33" s="10" t="inlineStr">
         <is>
@@ -3217,7 +3217,7 @@
         </is>
       </c>
       <c r="K34" s="7" t="n">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="L34" s="7" t="inlineStr">
         <is>
@@ -3280,7 +3280,7 @@
         </is>
       </c>
       <c r="K35" s="10" t="n">
-        <v>16</v>
+        <v>54</v>
       </c>
       <c r="L35" s="10" t="inlineStr">
         <is>
@@ -3343,7 +3343,7 @@
         </is>
       </c>
       <c r="K36" s="7" t="n">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="L36" s="7" t="inlineStr">
         <is>
@@ -3406,7 +3406,7 @@
         </is>
       </c>
       <c r="K37" s="10" t="n">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="L37" s="10" t="inlineStr">
         <is>
@@ -3469,7 +3469,7 @@
         </is>
       </c>
       <c r="K38" s="7" t="n">
-        <v>15</v>
+        <v>34</v>
       </c>
       <c r="L38" s="7" t="inlineStr">
         <is>
@@ -3532,7 +3532,7 @@
         </is>
       </c>
       <c r="K39" s="10" t="n">
-        <v>30</v>
+        <v>46</v>
       </c>
       <c r="L39" s="10" t="inlineStr">
         <is>
@@ -3595,7 +3595,7 @@
         </is>
       </c>
       <c r="K40" s="7" t="n">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="L40" s="7" t="inlineStr">
         <is>
@@ -3658,7 +3658,7 @@
         </is>
       </c>
       <c r="K41" s="10" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="L41" s="10" t="inlineStr">
         <is>
@@ -3721,7 +3721,7 @@
         </is>
       </c>
       <c r="K42" s="7" t="n">
-        <v>49</v>
+        <v>28</v>
       </c>
       <c r="L42" s="7" t="inlineStr">
         <is>
@@ -3784,7 +3784,7 @@
         </is>
       </c>
       <c r="K43" s="10" t="n">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="L43" s="10" t="inlineStr">
         <is>
@@ -3847,7 +3847,7 @@
         </is>
       </c>
       <c r="K44" s="7" t="n">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="L44" s="7" t="inlineStr">
         <is>
@@ -3910,7 +3910,7 @@
         </is>
       </c>
       <c r="K45" s="10" t="n">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="L45" s="10" t="inlineStr">
         <is>
@@ -3973,7 +3973,7 @@
         </is>
       </c>
       <c r="K46" s="7" t="n">
-        <v>22</v>
+        <v>49</v>
       </c>
       <c r="L46" s="7" t="inlineStr">
         <is>
@@ -4036,7 +4036,7 @@
         </is>
       </c>
       <c r="K47" s="10" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="L47" s="10" t="inlineStr">
         <is>
@@ -4099,7 +4099,7 @@
         </is>
       </c>
       <c r="K48" s="7" t="n">
-        <v>37</v>
+        <v>52</v>
       </c>
       <c r="L48" s="7" t="inlineStr">
         <is>
@@ -4162,7 +4162,7 @@
         </is>
       </c>
       <c r="K49" s="10" t="n">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="L49" s="10" t="inlineStr">
         <is>
@@ -4225,7 +4225,7 @@
         </is>
       </c>
       <c r="K50" s="7" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="L50" s="7" t="inlineStr">
         <is>
@@ -4288,7 +4288,7 @@
         </is>
       </c>
       <c r="K51" s="10" t="n">
-        <v>18</v>
+        <v>52</v>
       </c>
       <c r="L51" s="10" t="inlineStr">
         <is>
@@ -4351,7 +4351,7 @@
         </is>
       </c>
       <c r="K52" s="7" t="n">
-        <v>55</v>
+        <v>17</v>
       </c>
       <c r="L52" s="7" t="inlineStr">
         <is>
@@ -4414,7 +4414,7 @@
         </is>
       </c>
       <c r="K53" s="10" t="n">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="L53" s="10" t="inlineStr">
         <is>
@@ -4477,7 +4477,7 @@
         </is>
       </c>
       <c r="K54" s="7" t="n">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="L54" s="7" t="inlineStr">
         <is>
@@ -4540,7 +4540,7 @@
         </is>
       </c>
       <c r="K55" s="10" t="n">
-        <v>47</v>
+        <v>24</v>
       </c>
       <c r="L55" s="10" t="inlineStr">
         <is>
@@ -4603,7 +4603,7 @@
         </is>
       </c>
       <c r="K56" s="7" t="n">
-        <v>31</v>
+        <v>56</v>
       </c>
       <c r="L56" s="7" t="inlineStr">
         <is>
@@ -4666,7 +4666,7 @@
         </is>
       </c>
       <c r="K57" s="10" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="L57" s="10" t="inlineStr">
         <is>
@@ -4729,7 +4729,7 @@
         </is>
       </c>
       <c r="K58" s="7" t="n">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="L58" s="7" t="inlineStr">
         <is>
@@ -4792,7 +4792,7 @@
         </is>
       </c>
       <c r="K59" s="10" t="n">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="L59" s="10" t="inlineStr">
         <is>
@@ -4855,7 +4855,7 @@
         </is>
       </c>
       <c r="K60" s="7" t="n">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="L60" s="7" t="inlineStr">
         <is>
@@ -4918,7 +4918,7 @@
         </is>
       </c>
       <c r="K61" s="10" t="n">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="L61" s="10" t="inlineStr">
         <is>
@@ -4981,7 +4981,7 @@
         </is>
       </c>
       <c r="K62" s="7" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="L62" s="7" t="inlineStr">
         <is>
@@ -5044,7 +5044,7 @@
         </is>
       </c>
       <c r="K63" s="10" t="n">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="L63" s="10" t="inlineStr">
         <is>
@@ -5107,7 +5107,7 @@
         </is>
       </c>
       <c r="K64" s="7" t="n">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="L64" s="7" t="inlineStr">
         <is>
@@ -5170,7 +5170,7 @@
         </is>
       </c>
       <c r="K65" s="10" t="n">
-        <v>57</v>
+        <v>40</v>
       </c>
       <c r="L65" s="10" t="inlineStr">
         <is>
@@ -5233,7 +5233,7 @@
         </is>
       </c>
       <c r="K66" s="7" t="n">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="L66" s="7" t="inlineStr">
         <is>
@@ -5296,7 +5296,7 @@
         </is>
       </c>
       <c r="K67" s="10" t="n">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="L67" s="10" t="inlineStr">
         <is>
@@ -5359,7 +5359,7 @@
         </is>
       </c>
       <c r="K68" s="7" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="L68" s="7" t="inlineStr">
         <is>
@@ -5422,7 +5422,7 @@
         </is>
       </c>
       <c r="K69" s="10" t="n">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="L69" s="10" t="inlineStr">
         <is>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="K70" s="7" t="n">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="L70" s="7" t="inlineStr">
         <is>
@@ -5611,7 +5611,7 @@
         </is>
       </c>
       <c r="K72" s="7" t="n">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="L72" s="7" t="inlineStr">
         <is>
@@ -5674,7 +5674,7 @@
         </is>
       </c>
       <c r="K73" s="10" t="n">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="L73" s="10" t="inlineStr">
         <is>
@@ -5737,7 +5737,7 @@
         </is>
       </c>
       <c r="K74" s="7" t="n">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="L74" s="7" t="inlineStr">
         <is>
@@ -5800,7 +5800,7 @@
         </is>
       </c>
       <c r="K75" s="10" t="n">
-        <v>19</v>
+        <v>44</v>
       </c>
       <c r="L75" s="10" t="inlineStr">
         <is>
@@ -5863,7 +5863,7 @@
         </is>
       </c>
       <c r="K76" s="7" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="L76" s="7" t="inlineStr">
         <is>
@@ -5926,7 +5926,7 @@
         </is>
       </c>
       <c r="K77" s="10" t="n">
-        <v>28</v>
+        <v>56</v>
       </c>
       <c r="L77" s="10" t="inlineStr">
         <is>
@@ -5989,7 +5989,7 @@
         </is>
       </c>
       <c r="K78" s="7" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="L78" s="7" t="inlineStr">
         <is>
@@ -6052,7 +6052,7 @@
         </is>
       </c>
       <c r="K79" s="10" t="n">
-        <v>58</v>
+        <v>20</v>
       </c>
       <c r="L79" s="10" t="inlineStr">
         <is>
@@ -6115,7 +6115,7 @@
         </is>
       </c>
       <c r="K80" s="7" t="n">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="L80" s="7" t="inlineStr">
         <is>
@@ -6178,7 +6178,7 @@
         </is>
       </c>
       <c r="K81" s="10" t="n">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="L81" s="10" t="inlineStr">
         <is>
@@ -6241,7 +6241,7 @@
         </is>
       </c>
       <c r="K82" s="7" t="n">
-        <v>24</v>
+        <v>44</v>
       </c>
       <c r="L82" s="7" t="inlineStr">
         <is>
@@ -6304,7 +6304,7 @@
         </is>
       </c>
       <c r="K83" s="10" t="n">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="L83" s="10" t="inlineStr">
         <is>
@@ -6367,7 +6367,7 @@
         </is>
       </c>
       <c r="K84" s="7" t="n">
-        <v>51</v>
+        <v>27</v>
       </c>
       <c r="L84" s="7" t="inlineStr">
         <is>
@@ -6430,7 +6430,7 @@
         </is>
       </c>
       <c r="K85" s="10" t="n">
-        <v>29</v>
+        <v>53</v>
       </c>
       <c r="L85" s="10" t="inlineStr">
         <is>
@@ -6493,7 +6493,7 @@
         </is>
       </c>
       <c r="K86" s="7" t="n">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="L86" s="7" t="inlineStr">
         <is>
@@ -6556,7 +6556,7 @@
         </is>
       </c>
       <c r="K87" s="10" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="L87" s="10" t="inlineStr">
         <is>
@@ -6619,7 +6619,7 @@
         </is>
       </c>
       <c r="K88" s="7" t="n">
-        <v>30</v>
+        <v>53</v>
       </c>
       <c r="L88" s="7" t="inlineStr">
         <is>
@@ -6682,7 +6682,7 @@
         </is>
       </c>
       <c r="K89" s="10" t="n">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="L89" s="10" t="inlineStr">
         <is>
@@ -6745,7 +6745,7 @@
         </is>
       </c>
       <c r="K90" s="7" t="n">
-        <v>33</v>
+        <v>55</v>
       </c>
       <c r="L90" s="7" t="inlineStr">
         <is>
@@ -6808,7 +6808,7 @@
         </is>
       </c>
       <c r="K91" s="10" t="n">
-        <v>27</v>
+        <v>56</v>
       </c>
       <c r="L91" s="10" t="inlineStr">
         <is>
@@ -6871,7 +6871,7 @@
         </is>
       </c>
       <c r="K92" s="7" t="n">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="L92" s="7" t="inlineStr">
         <is>
@@ -6934,7 +6934,7 @@
         </is>
       </c>
       <c r="K93" s="10" t="n">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="L93" s="10" t="inlineStr">
         <is>
@@ -6997,7 +6997,7 @@
         </is>
       </c>
       <c r="K94" s="7" t="n">
-        <v>20</v>
+        <v>54</v>
       </c>
       <c r="L94" s="7" t="inlineStr">
         <is>
@@ -7060,7 +7060,7 @@
         </is>
       </c>
       <c r="K95" s="10" t="n">
-        <v>54</v>
+        <v>30</v>
       </c>
       <c r="L95" s="10" t="inlineStr">
         <is>
@@ -7123,7 +7123,7 @@
         </is>
       </c>
       <c r="K96" s="7" t="n">
-        <v>31</v>
+        <v>43</v>
       </c>
       <c r="L96" s="7" t="inlineStr">
         <is>
@@ -7186,7 +7186,7 @@
         </is>
       </c>
       <c r="K97" s="10" t="n">
-        <v>50</v>
+        <v>19</v>
       </c>
       <c r="L97" s="10" t="inlineStr">
         <is>
@@ -7249,7 +7249,7 @@
         </is>
       </c>
       <c r="K98" s="7" t="n">
-        <v>19</v>
+        <v>44</v>
       </c>
       <c r="L98" s="7" t="inlineStr">
         <is>
@@ -7312,7 +7312,7 @@
         </is>
       </c>
       <c r="K99" s="10" t="n">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="L99" s="10" t="inlineStr">
         <is>
@@ -7375,7 +7375,7 @@
         </is>
       </c>
       <c r="K100" s="7" t="n">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="L100" s="7" t="inlineStr">
         <is>
@@ -7438,7 +7438,7 @@
         </is>
       </c>
       <c r="K101" s="10" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="L101" s="10" t="inlineStr">
         <is>
@@ -7501,7 +7501,7 @@
         </is>
       </c>
       <c r="K102" s="7" t="n">
-        <v>29</v>
+        <v>46</v>
       </c>
       <c r="L102" s="7" t="inlineStr">
         <is>
@@ -7564,7 +7564,7 @@
         </is>
       </c>
       <c r="K103" s="10" t="n">
-        <v>28</v>
+        <v>44</v>
       </c>
       <c r="L103" s="10" t="inlineStr">
         <is>
@@ -7627,7 +7627,7 @@
         </is>
       </c>
       <c r="K104" s="7" t="n">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="L104" s="7" t="inlineStr">
         <is>
@@ -7690,7 +7690,7 @@
         </is>
       </c>
       <c r="K105" s="10" t="n">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="L105" s="10" t="inlineStr">
         <is>
@@ -7753,7 +7753,7 @@
         </is>
       </c>
       <c r="K106" s="7" t="n">
-        <v>22</v>
+        <v>54</v>
       </c>
       <c r="L106" s="7" t="inlineStr">
         <is>
@@ -7816,7 +7816,7 @@
         </is>
       </c>
       <c r="K107" s="10" t="n">
-        <v>55</v>
+        <v>42</v>
       </c>
       <c r="L107" s="10" t="inlineStr">
         <is>
@@ -7879,7 +7879,7 @@
         </is>
       </c>
       <c r="K108" s="7" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="L108" s="7" t="inlineStr">
         <is>
@@ -7942,7 +7942,7 @@
         </is>
       </c>
       <c r="K109" s="10" t="n">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="L109" s="10" t="inlineStr">
         <is>
@@ -8005,7 +8005,7 @@
         </is>
       </c>
       <c r="K110" s="7" t="n">
-        <v>41</v>
+        <v>23</v>
       </c>
       <c r="L110" s="7" t="inlineStr">
         <is>
@@ -8068,7 +8068,7 @@
         </is>
       </c>
       <c r="K111" s="10" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="L111" s="10" t="inlineStr">
         <is>
@@ -8131,7 +8131,7 @@
         </is>
       </c>
       <c r="K112" s="7" t="n">
-        <v>56</v>
+        <v>20</v>
       </c>
       <c r="L112" s="7" t="inlineStr">
         <is>
@@ -8194,7 +8194,7 @@
         </is>
       </c>
       <c r="K113" s="10" t="n">
-        <v>53</v>
+        <v>17</v>
       </c>
       <c r="L113" s="10" t="inlineStr">
         <is>
@@ -8257,7 +8257,7 @@
         </is>
       </c>
       <c r="K114" s="7" t="n">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="L114" s="7" t="inlineStr">
         <is>
@@ -8320,7 +8320,7 @@
         </is>
       </c>
       <c r="K115" s="10" t="n">
-        <v>58</v>
+        <v>15</v>
       </c>
       <c r="L115" s="10" t="inlineStr">
         <is>
@@ -8383,7 +8383,7 @@
         </is>
       </c>
       <c r="K116" s="7" t="n">
-        <v>53</v>
+        <v>19</v>
       </c>
       <c r="L116" s="7" t="inlineStr">
         <is>
@@ -8446,7 +8446,7 @@
         </is>
       </c>
       <c r="K117" s="10" t="n">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="L117" s="10" t="inlineStr">
         <is>
@@ -8509,7 +8509,7 @@
         </is>
       </c>
       <c r="K118" s="7" t="n">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="L118" s="7" t="inlineStr">
         <is>
@@ -8572,7 +8572,7 @@
         </is>
       </c>
       <c r="K119" s="10" t="n">
-        <v>46</v>
+        <v>21</v>
       </c>
       <c r="L119" s="10" t="inlineStr">
         <is>
@@ -8635,7 +8635,7 @@
         </is>
       </c>
       <c r="K120" s="7" t="n">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="L120" s="7" t="inlineStr">
         <is>
@@ -8698,7 +8698,7 @@
         </is>
       </c>
       <c r="K121" s="10" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="L121" s="10" t="inlineStr">
         <is>
@@ -8761,7 +8761,7 @@
         </is>
       </c>
       <c r="K122" s="7" t="n">
-        <v>18</v>
+        <v>47</v>
       </c>
       <c r="L122" s="7" t="inlineStr">
         <is>
@@ -8824,7 +8824,7 @@
         </is>
       </c>
       <c r="K123" s="10" t="n">
-        <v>58</v>
+        <v>21</v>
       </c>
       <c r="L123" s="10" t="inlineStr">
         <is>
@@ -8887,7 +8887,7 @@
         </is>
       </c>
       <c r="K124" s="7" t="n">
-        <v>54</v>
+        <v>15</v>
       </c>
       <c r="L124" s="7" t="inlineStr">
         <is>
@@ -8950,7 +8950,7 @@
         </is>
       </c>
       <c r="K125" s="10" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="L125" s="10" t="inlineStr">
         <is>
@@ -9013,7 +9013,7 @@
         </is>
       </c>
       <c r="K126" s="7" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="L126" s="7" t="inlineStr">
         <is>
@@ -9076,7 +9076,7 @@
         </is>
       </c>
       <c r="K127" s="10" t="n">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="L127" s="10" t="inlineStr">
         <is>
@@ -9139,7 +9139,7 @@
         </is>
       </c>
       <c r="K128" s="7" t="n">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="L128" s="7" t="inlineStr">
         <is>
@@ -9202,7 +9202,7 @@
         </is>
       </c>
       <c r="K129" s="10" t="n">
-        <v>25</v>
+        <v>48</v>
       </c>
       <c r="L129" s="10" t="inlineStr">
         <is>
@@ -9265,7 +9265,7 @@
         </is>
       </c>
       <c r="K130" s="7" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="L130" s="7" t="inlineStr">
         <is>
@@ -9328,7 +9328,7 @@
         </is>
       </c>
       <c r="K131" s="10" t="n">
-        <v>21</v>
+        <v>40</v>
       </c>
       <c r="L131" s="10" t="inlineStr">
         <is>
@@ -9391,7 +9391,7 @@
         </is>
       </c>
       <c r="K132" s="7" t="n">
-        <v>54</v>
+        <v>41</v>
       </c>
       <c r="L132" s="7" t="inlineStr">
         <is>
@@ -9454,7 +9454,7 @@
         </is>
       </c>
       <c r="K133" s="10" t="n">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="L133" s="10" t="inlineStr">
         <is>
@@ -9517,7 +9517,7 @@
         </is>
       </c>
       <c r="K134" s="7" t="n">
-        <v>41</v>
+        <v>17</v>
       </c>
       <c r="L134" s="7" t="inlineStr">
         <is>
@@ -9580,7 +9580,7 @@
         </is>
       </c>
       <c r="K135" s="10" t="n">
-        <v>46</v>
+        <v>20</v>
       </c>
       <c r="L135" s="10" t="inlineStr">
         <is>
@@ -9643,7 +9643,7 @@
         </is>
       </c>
       <c r="K136" s="7" t="n">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="L136" s="7" t="inlineStr">
         <is>
@@ -9706,7 +9706,7 @@
         </is>
       </c>
       <c r="K137" s="10" t="n">
-        <v>54</v>
+        <v>26</v>
       </c>
       <c r="L137" s="10" t="inlineStr">
         <is>
@@ -9769,7 +9769,7 @@
         </is>
       </c>
       <c r="K138" s="7" t="n">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="L138" s="7" t="inlineStr">
         <is>
@@ -9832,7 +9832,7 @@
         </is>
       </c>
       <c r="K139" s="10" t="n">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="L139" s="10" t="inlineStr">
         <is>
@@ -9895,7 +9895,7 @@
         </is>
       </c>
       <c r="K140" s="7" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="L140" s="7" t="inlineStr">
         <is>
@@ -9958,7 +9958,7 @@
         </is>
       </c>
       <c r="K141" s="10" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="L141" s="10" t="inlineStr">
         <is>
@@ -10021,7 +10021,7 @@
         </is>
       </c>
       <c r="K142" s="7" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="L142" s="7" t="inlineStr">
         <is>
@@ -10084,7 +10084,7 @@
         </is>
       </c>
       <c r="K143" s="10" t="n">
-        <v>30</v>
+        <v>54</v>
       </c>
       <c r="L143" s="10" t="inlineStr">
         <is>
@@ -10147,7 +10147,7 @@
         </is>
       </c>
       <c r="K144" s="7" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="L144" s="7" t="inlineStr">
         <is>
@@ -10210,7 +10210,7 @@
         </is>
       </c>
       <c r="K145" s="10" t="n">
-        <v>57</v>
+        <v>21</v>
       </c>
       <c r="L145" s="10" t="inlineStr">
         <is>
@@ -10273,7 +10273,7 @@
         </is>
       </c>
       <c r="K146" s="7" t="n">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="L146" s="7" t="inlineStr">
         <is>
@@ -10336,7 +10336,7 @@
         </is>
       </c>
       <c r="K147" s="10" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="L147" s="10" t="inlineStr">
         <is>
@@ -10399,7 +10399,7 @@
         </is>
       </c>
       <c r="K148" s="7" t="n">
-        <v>58</v>
+        <v>16</v>
       </c>
       <c r="L148" s="7" t="inlineStr">
         <is>
@@ -10462,7 +10462,7 @@
         </is>
       </c>
       <c r="K149" s="10" t="n">
-        <v>38</v>
+        <v>55</v>
       </c>
       <c r="L149" s="10" t="inlineStr">
         <is>
@@ -10525,7 +10525,7 @@
         </is>
       </c>
       <c r="K150" s="7" t="n">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="L150" s="7" t="inlineStr">
         <is>
@@ -10588,7 +10588,7 @@
         </is>
       </c>
       <c r="K151" s="10" t="n">
-        <v>20</v>
+        <v>37</v>
       </c>
       <c r="L151" s="10" t="inlineStr">
         <is>
@@ -10651,7 +10651,7 @@
         </is>
       </c>
       <c r="K152" s="7" t="n">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="L152" s="7" t="inlineStr">
         <is>
@@ -10714,7 +10714,7 @@
         </is>
       </c>
       <c r="K153" s="10" t="n">
-        <v>32</v>
+        <v>54</v>
       </c>
       <c r="L153" s="10" t="inlineStr">
         <is>
@@ -10777,7 +10777,7 @@
         </is>
       </c>
       <c r="K154" s="7" t="n">
-        <v>50</v>
+        <v>22</v>
       </c>
       <c r="L154" s="7" t="inlineStr">
         <is>
@@ -10840,7 +10840,7 @@
         </is>
       </c>
       <c r="K155" s="10" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="L155" s="10" t="inlineStr">
         <is>
@@ -10966,7 +10966,7 @@
         </is>
       </c>
       <c r="K157" s="10" t="n">
-        <v>44</v>
+        <v>29</v>
       </c>
       <c r="L157" s="10" t="inlineStr">
         <is>
@@ -11029,7 +11029,7 @@
         </is>
       </c>
       <c r="K158" s="7" t="n">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="L158" s="7" t="inlineStr">
         <is>
@@ -11092,7 +11092,7 @@
         </is>
       </c>
       <c r="K159" s="10" t="n">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="L159" s="10" t="inlineStr">
         <is>
@@ -11155,7 +11155,7 @@
         </is>
       </c>
       <c r="K160" s="7" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="L160" s="7" t="inlineStr">
         <is>
@@ -11218,7 +11218,7 @@
         </is>
       </c>
       <c r="K161" s="10" t="n">
-        <v>19</v>
+        <v>56</v>
       </c>
       <c r="L161" s="10" t="inlineStr">
         <is>
@@ -11281,7 +11281,7 @@
         </is>
       </c>
       <c r="K162" s="7" t="n">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="L162" s="7" t="inlineStr">
         <is>
@@ -11344,7 +11344,7 @@
         </is>
       </c>
       <c r="K163" s="10" t="n">
-        <v>54</v>
+        <v>20</v>
       </c>
       <c r="L163" s="10" t="inlineStr">
         <is>
@@ -11407,7 +11407,7 @@
         </is>
       </c>
       <c r="K164" s="7" t="n">
-        <v>49</v>
+        <v>28</v>
       </c>
       <c r="L164" s="7" t="inlineStr">
         <is>
@@ -11470,7 +11470,7 @@
         </is>
       </c>
       <c r="K165" s="10" t="n">
-        <v>54</v>
+        <v>40</v>
       </c>
       <c r="L165" s="10" t="inlineStr">
         <is>
@@ -11533,7 +11533,7 @@
         </is>
       </c>
       <c r="K166" s="7" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="L166" s="7" t="inlineStr">
         <is>
@@ -11596,7 +11596,7 @@
         </is>
       </c>
       <c r="K167" s="10" t="n">
-        <v>21</v>
+        <v>48</v>
       </c>
       <c r="L167" s="10" t="inlineStr">
         <is>
@@ -11659,7 +11659,7 @@
         </is>
       </c>
       <c r="K168" s="7" t="n">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="L168" s="7" t="inlineStr">
         <is>
@@ -11722,7 +11722,7 @@
         </is>
       </c>
       <c r="K169" s="10" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="L169" s="10" t="inlineStr">
         <is>
@@ -11785,7 +11785,7 @@
         </is>
       </c>
       <c r="K170" s="7" t="n">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="L170" s="7" t="inlineStr">
         <is>
@@ -11848,7 +11848,7 @@
         </is>
       </c>
       <c r="K171" s="10" t="n">
-        <v>49</v>
+        <v>15</v>
       </c>
       <c r="L171" s="10" t="inlineStr">
         <is>
@@ -11911,7 +11911,7 @@
         </is>
       </c>
       <c r="K172" s="7" t="n">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="L172" s="7" t="inlineStr">
         <is>
@@ -11974,7 +11974,7 @@
         </is>
       </c>
       <c r="K173" s="10" t="n">
-        <v>44</v>
+        <v>23</v>
       </c>
       <c r="L173" s="10" t="inlineStr">
         <is>
@@ -12037,7 +12037,7 @@
         </is>
       </c>
       <c r="K174" s="7" t="n">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="L174" s="7" t="inlineStr">
         <is>
@@ -12100,7 +12100,7 @@
         </is>
       </c>
       <c r="K175" s="10" t="n">
-        <v>33</v>
+        <v>51</v>
       </c>
       <c r="L175" s="10" t="inlineStr">
         <is>
@@ -12163,7 +12163,7 @@
         </is>
       </c>
       <c r="K176" s="7" t="n">
-        <v>28</v>
+        <v>47</v>
       </c>
       <c r="L176" s="7" t="inlineStr">
         <is>
@@ -12226,7 +12226,7 @@
         </is>
       </c>
       <c r="K177" s="10" t="n">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="L177" s="10" t="inlineStr">
         <is>
@@ -12289,7 +12289,7 @@
         </is>
       </c>
       <c r="K178" s="7" t="n">
-        <v>19</v>
+        <v>36</v>
       </c>
       <c r="L178" s="7" t="inlineStr">
         <is>
@@ -12352,7 +12352,7 @@
         </is>
       </c>
       <c r="K179" s="10" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="L179" s="10" t="inlineStr">
         <is>
@@ -12415,7 +12415,7 @@
         </is>
       </c>
       <c r="K180" s="7" t="n">
-        <v>34</v>
+        <v>48</v>
       </c>
       <c r="L180" s="7" t="inlineStr">
         <is>
@@ -12478,7 +12478,7 @@
         </is>
       </c>
       <c r="K181" s="10" t="n">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="L181" s="10" t="inlineStr">
         <is>
@@ -12541,7 +12541,7 @@
         </is>
       </c>
       <c r="K182" s="7" t="n">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="L182" s="7" t="inlineStr">
         <is>
@@ -12604,7 +12604,7 @@
         </is>
       </c>
       <c r="K183" s="10" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="L183" s="10" t="inlineStr">
         <is>
@@ -12667,7 +12667,7 @@
         </is>
       </c>
       <c r="K184" s="7" t="n">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="L184" s="7" t="inlineStr">
         <is>
@@ -12730,7 +12730,7 @@
         </is>
       </c>
       <c r="K185" s="10" t="n">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="L185" s="10" t="inlineStr">
         <is>
@@ -12793,7 +12793,7 @@
         </is>
       </c>
       <c r="K186" s="7" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="L186" s="7" t="inlineStr">
         <is>
@@ -12856,7 +12856,7 @@
         </is>
       </c>
       <c r="K187" s="10" t="n">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="L187" s="10" t="inlineStr">
         <is>
@@ -12919,7 +12919,7 @@
         </is>
       </c>
       <c r="K188" s="7" t="n">
-        <v>31</v>
+        <v>57</v>
       </c>
       <c r="L188" s="7" t="inlineStr">
         <is>
@@ -12982,7 +12982,7 @@
         </is>
       </c>
       <c r="K189" s="10" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="L189" s="10" t="inlineStr">
         <is>
@@ -13045,7 +13045,7 @@
         </is>
       </c>
       <c r="K190" s="7" t="n">
-        <v>27</v>
+        <v>54</v>
       </c>
       <c r="L190" s="7" t="inlineStr">
         <is>
@@ -13108,7 +13108,7 @@
         </is>
       </c>
       <c r="K191" s="10" t="n">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="L191" s="10" t="inlineStr">
         <is>
@@ -13171,7 +13171,7 @@
         </is>
       </c>
       <c r="K192" s="7" t="n">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="L192" s="7" t="inlineStr">
         <is>
@@ -13234,7 +13234,7 @@
         </is>
       </c>
       <c r="K193" s="10" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="L193" s="10" t="inlineStr">
         <is>
@@ -13297,7 +13297,7 @@
         </is>
       </c>
       <c r="K194" s="7" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="L194" s="7" t="inlineStr">
         <is>
@@ -13360,7 +13360,7 @@
         </is>
       </c>
       <c r="K195" s="10" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="L195" s="10" t="inlineStr">
         <is>
@@ -13423,7 +13423,7 @@
         </is>
       </c>
       <c r="K196" s="7" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="L196" s="7" t="inlineStr">
         <is>
@@ -13486,7 +13486,7 @@
         </is>
       </c>
       <c r="K197" s="10" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="L197" s="10" t="inlineStr">
         <is>
@@ -13549,7 +13549,7 @@
         </is>
       </c>
       <c r="K198" s="7" t="n">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="L198" s="7" t="inlineStr">
         <is>
@@ -13612,7 +13612,7 @@
         </is>
       </c>
       <c r="K199" s="10" t="n">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="L199" s="10" t="inlineStr">
         <is>
@@ -13675,7 +13675,7 @@
         </is>
       </c>
       <c r="K200" s="7" t="n">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="L200" s="7" t="inlineStr">
         <is>
@@ -13738,7 +13738,7 @@
         </is>
       </c>
       <c r="K201" s="10" t="n">
-        <v>20</v>
+        <v>42</v>
       </c>
       <c r="L201" s="10" t="inlineStr">
         <is>
@@ -13801,7 +13801,7 @@
         </is>
       </c>
       <c r="K202" s="7" t="n">
-        <v>48</v>
+        <v>21</v>
       </c>
       <c r="L202" s="7" t="inlineStr">
         <is>
@@ -13927,7 +13927,7 @@
         </is>
       </c>
       <c r="K204" s="7" t="n">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="L204" s="7" t="inlineStr">
         <is>
@@ -13990,7 +13990,7 @@
         </is>
       </c>
       <c r="K205" s="10" t="n">
-        <v>49</v>
+        <v>20</v>
       </c>
       <c r="L205" s="10" t="inlineStr">
         <is>
@@ -14053,7 +14053,7 @@
         </is>
       </c>
       <c r="K206" s="7" t="n">
-        <v>18</v>
+        <v>47</v>
       </c>
       <c r="L206" s="7" t="inlineStr">
         <is>
@@ -14116,7 +14116,7 @@
         </is>
       </c>
       <c r="K207" s="10" t="n">
-        <v>47</v>
+        <v>28</v>
       </c>
       <c r="L207" s="10" t="inlineStr">
         <is>
@@ -14179,7 +14179,7 @@
         </is>
       </c>
       <c r="K208" s="7" t="n">
-        <v>20</v>
+        <v>51</v>
       </c>
       <c r="L208" s="7" t="inlineStr">
         <is>
@@ -14242,7 +14242,7 @@
         </is>
       </c>
       <c r="K209" s="10" t="n">
-        <v>46</v>
+        <v>30</v>
       </c>
       <c r="L209" s="10" t="inlineStr">
         <is>
@@ -14305,7 +14305,7 @@
         </is>
       </c>
       <c r="K210" s="7" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="L210" s="7" t="inlineStr">
         <is>
@@ -14368,7 +14368,7 @@
         </is>
       </c>
       <c r="K211" s="10" t="n">
-        <v>49</v>
+        <v>28</v>
       </c>
       <c r="L211" s="10" t="inlineStr">
         <is>
@@ -14431,7 +14431,7 @@
         </is>
       </c>
       <c r="K212" s="7" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="L212" s="7" t="inlineStr">
         <is>
@@ -14494,7 +14494,7 @@
         </is>
       </c>
       <c r="K213" s="10" t="n">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="L213" s="10" t="inlineStr">
         <is>
@@ -14557,7 +14557,7 @@
         </is>
       </c>
       <c r="K214" s="7" t="n">
-        <v>56</v>
+        <v>37</v>
       </c>
       <c r="L214" s="7" t="inlineStr">
         <is>
@@ -14620,7 +14620,7 @@
         </is>
       </c>
       <c r="K215" s="10" t="n">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="L215" s="10" t="inlineStr">
         <is>
@@ -14683,7 +14683,7 @@
         </is>
       </c>
       <c r="K216" s="7" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="L216" s="7" t="inlineStr">
         <is>
@@ -14746,7 +14746,7 @@
         </is>
       </c>
       <c r="K217" s="10" t="n">
-        <v>51</v>
+        <v>19</v>
       </c>
       <c r="L217" s="10" t="inlineStr">
         <is>
@@ -14809,7 +14809,7 @@
         </is>
       </c>
       <c r="K218" s="7" t="n">
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="L218" s="7" t="inlineStr">
         <is>
@@ -14872,7 +14872,7 @@
         </is>
       </c>
       <c r="K219" s="10" t="n">
-        <v>46</v>
+        <v>15</v>
       </c>
       <c r="L219" s="10" t="inlineStr">
         <is>
@@ -14935,7 +14935,7 @@
         </is>
       </c>
       <c r="K220" s="7" t="n">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="L220" s="7" t="inlineStr">
         <is>
@@ -15061,7 +15061,7 @@
         </is>
       </c>
       <c r="K222" s="7" t="n">
-        <v>24</v>
+        <v>42</v>
       </c>
       <c r="L222" s="7" t="inlineStr">
         <is>
@@ -15124,7 +15124,7 @@
         </is>
       </c>
       <c r="K223" s="10" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="L223" s="10" t="inlineStr">
         <is>
@@ -15187,7 +15187,7 @@
         </is>
       </c>
       <c r="K224" s="7" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="L224" s="7" t="inlineStr">
         <is>
@@ -15250,7 +15250,7 @@
         </is>
       </c>
       <c r="K225" s="10" t="n">
-        <v>27</v>
+        <v>53</v>
       </c>
       <c r="L225" s="10" t="inlineStr">
         <is>
@@ -15313,7 +15313,7 @@
         </is>
       </c>
       <c r="K226" s="7" t="n">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="L226" s="7" t="inlineStr">
         <is>
@@ -15376,7 +15376,7 @@
         </is>
       </c>
       <c r="K227" s="10" t="n">
-        <v>56</v>
+        <v>44</v>
       </c>
       <c r="L227" s="10" t="inlineStr">
         <is>
@@ -15439,7 +15439,7 @@
         </is>
       </c>
       <c r="K228" s="7" t="n">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="L228" s="7" t="inlineStr">
         <is>
@@ -15502,7 +15502,7 @@
         </is>
       </c>
       <c r="K229" s="10" t="n">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="L229" s="10" t="inlineStr">
         <is>
@@ -15565,7 +15565,7 @@
         </is>
       </c>
       <c r="K230" s="7" t="n">
-        <v>57</v>
+        <v>18</v>
       </c>
       <c r="L230" s="7" t="inlineStr">
         <is>
@@ -15628,7 +15628,7 @@
         </is>
       </c>
       <c r="K231" s="10" t="n">
-        <v>33</v>
+        <v>56</v>
       </c>
       <c r="L231" s="10" t="inlineStr">
         <is>
@@ -15691,7 +15691,7 @@
         </is>
       </c>
       <c r="K232" s="7" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="L232" s="7" t="inlineStr">
         <is>
@@ -15754,7 +15754,7 @@
         </is>
       </c>
       <c r="K233" s="10" t="n">
-        <v>57</v>
+        <v>32</v>
       </c>
       <c r="L233" s="10" t="inlineStr">
         <is>
@@ -15817,7 +15817,7 @@
         </is>
       </c>
       <c r="K234" s="7" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="L234" s="7" t="inlineStr">
         <is>
@@ -15880,7 +15880,7 @@
         </is>
       </c>
       <c r="K235" s="10" t="n">
-        <v>33</v>
+        <v>48</v>
       </c>
       <c r="L235" s="10" t="inlineStr">
         <is>
@@ -15943,7 +15943,7 @@
         </is>
       </c>
       <c r="K236" s="7" t="n">
-        <v>58</v>
+        <v>23</v>
       </c>
       <c r="L236" s="7" t="inlineStr">
         <is>
@@ -16069,7 +16069,7 @@
         </is>
       </c>
       <c r="K238" s="7" t="n">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="L238" s="7" t="inlineStr">
         <is>
@@ -16132,7 +16132,7 @@
         </is>
       </c>
       <c r="K239" s="10" t="n">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="L239" s="10" t="inlineStr">
         <is>
@@ -16195,7 +16195,7 @@
         </is>
       </c>
       <c r="K240" s="7" t="n">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="L240" s="7" t="inlineStr">
         <is>
@@ -16258,7 +16258,7 @@
         </is>
       </c>
       <c r="K241" s="10" t="n">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="L241" s="10" t="inlineStr">
         <is>
@@ -16321,7 +16321,7 @@
         </is>
       </c>
       <c r="K242" s="7" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="L242" s="7" t="inlineStr">
         <is>
@@ -16384,7 +16384,7 @@
         </is>
       </c>
       <c r="K243" s="10" t="n">
-        <v>33</v>
+        <v>47</v>
       </c>
       <c r="L243" s="10" t="inlineStr">
         <is>
@@ -16447,7 +16447,7 @@
         </is>
       </c>
       <c r="K244" s="7" t="n">
-        <v>25</v>
+        <v>54</v>
       </c>
       <c r="L244" s="7" t="inlineStr">
         <is>
@@ -16510,7 +16510,7 @@
         </is>
       </c>
       <c r="K245" s="10" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="L245" s="10" t="inlineStr">
         <is>
@@ -16573,7 +16573,7 @@
         </is>
       </c>
       <c r="K246" s="7" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="L246" s="7" t="inlineStr">
         <is>
@@ -16636,7 +16636,7 @@
         </is>
       </c>
       <c r="K247" s="10" t="n">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="L247" s="10" t="inlineStr">
         <is>
@@ -16699,7 +16699,7 @@
         </is>
       </c>
       <c r="K248" s="7" t="n">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="L248" s="7" t="inlineStr">
         <is>
@@ -16762,7 +16762,7 @@
         </is>
       </c>
       <c r="K249" s="10" t="n">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="L249" s="10" t="inlineStr">
         <is>
@@ -16825,7 +16825,7 @@
         </is>
       </c>
       <c r="K250" s="7" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="L250" s="7" t="inlineStr">
         <is>
@@ -16888,7 +16888,7 @@
         </is>
       </c>
       <c r="K251" s="10" t="n">
-        <v>19</v>
+        <v>36</v>
       </c>
       <c r="L251" s="10" t="inlineStr">
         <is>
@@ -16951,7 +16951,7 @@
         </is>
       </c>
       <c r="K252" s="7" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="L252" s="7" t="inlineStr">
         <is>
@@ -17014,7 +17014,7 @@
         </is>
       </c>
       <c r="K253" s="10" t="n">
-        <v>17</v>
+        <v>35</v>
       </c>
       <c r="L253" s="10" t="inlineStr">
         <is>
@@ -17077,7 +17077,7 @@
         </is>
       </c>
       <c r="K254" s="7" t="n">
-        <v>55</v>
+        <v>38</v>
       </c>
       <c r="L254" s="7" t="inlineStr">
         <is>
@@ -17140,7 +17140,7 @@
         </is>
       </c>
       <c r="K255" s="10" t="n">
-        <v>45</v>
+        <v>56</v>
       </c>
       <c r="L255" s="10" t="inlineStr">
         <is>
@@ -17266,7 +17266,7 @@
         </is>
       </c>
       <c r="K257" s="10" t="n">
-        <v>55</v>
+        <v>27</v>
       </c>
       <c r="L257" s="10" t="inlineStr">
         <is>
@@ -17329,7 +17329,7 @@
         </is>
       </c>
       <c r="K258" s="7" t="n">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="L258" s="7" t="inlineStr">
         <is>
@@ -17392,7 +17392,7 @@
         </is>
       </c>
       <c r="K259" s="10" t="n">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="L259" s="10" t="inlineStr">
         <is>
@@ -17455,7 +17455,7 @@
         </is>
       </c>
       <c r="K260" s="7" t="n">
-        <v>23</v>
+        <v>55</v>
       </c>
       <c r="L260" s="7" t="inlineStr">
         <is>
@@ -17518,7 +17518,7 @@
         </is>
       </c>
       <c r="K261" s="10" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="L261" s="10" t="inlineStr">
         <is>
@@ -17581,7 +17581,7 @@
         </is>
       </c>
       <c r="K262" s="7" t="n">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="L262" s="7" t="inlineStr">
         <is>
@@ -17644,7 +17644,7 @@
         </is>
       </c>
       <c r="K263" s="10" t="n">
-        <v>55</v>
+        <v>44</v>
       </c>
       <c r="L263" s="10" t="inlineStr">
         <is>
@@ -17707,7 +17707,7 @@
         </is>
       </c>
       <c r="K264" s="7" t="n">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="L264" s="7" t="inlineStr">
         <is>
@@ -17770,7 +17770,7 @@
         </is>
       </c>
       <c r="K265" s="10" t="n">
-        <v>19</v>
+        <v>47</v>
       </c>
       <c r="L265" s="10" t="inlineStr">
         <is>
@@ -17833,7 +17833,7 @@
         </is>
       </c>
       <c r="K266" s="7" t="n">
-        <v>39</v>
+        <v>18</v>
       </c>
       <c r="L266" s="7" t="inlineStr">
         <is>
@@ -17896,7 +17896,7 @@
         </is>
       </c>
       <c r="K267" s="10" t="n">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="L267" s="10" t="inlineStr">
         <is>
@@ -17959,7 +17959,7 @@
         </is>
       </c>
       <c r="K268" s="7" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="L268" s="7" t="inlineStr">
         <is>
@@ -18022,7 +18022,7 @@
         </is>
       </c>
       <c r="K269" s="10" t="n">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="L269" s="10" t="inlineStr">
         <is>
@@ -18085,7 +18085,7 @@
         </is>
       </c>
       <c r="K270" s="7" t="n">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="L270" s="7" t="inlineStr">
         <is>
@@ -18148,7 +18148,7 @@
         </is>
       </c>
       <c r="K271" s="10" t="n">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="L271" s="10" t="inlineStr">
         <is>
@@ -18211,7 +18211,7 @@
         </is>
       </c>
       <c r="K272" s="7" t="n">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="L272" s="7" t="inlineStr">
         <is>
@@ -18274,7 +18274,7 @@
         </is>
       </c>
       <c r="K273" s="10" t="n">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="L273" s="10" t="inlineStr">
         <is>
@@ -18337,7 +18337,7 @@
         </is>
       </c>
       <c r="K274" s="7" t="n">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="L274" s="7" t="inlineStr">
         <is>
@@ -18400,7 +18400,7 @@
         </is>
       </c>
       <c r="K275" s="10" t="n">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="L275" s="10" t="inlineStr">
         <is>
@@ -18463,7 +18463,7 @@
         </is>
       </c>
       <c r="K276" s="7" t="n">
-        <v>40</v>
+        <v>18</v>
       </c>
       <c r="L276" s="7" t="inlineStr">
         <is>
@@ -18526,7 +18526,7 @@
         </is>
       </c>
       <c r="K277" s="10" t="n">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="L277" s="10" t="inlineStr">
         <is>
@@ -18589,7 +18589,7 @@
         </is>
       </c>
       <c r="K278" s="7" t="n">
-        <v>24</v>
+        <v>51</v>
       </c>
       <c r="L278" s="7" t="inlineStr">
         <is>
@@ -18652,7 +18652,7 @@
         </is>
       </c>
       <c r="K279" s="10" t="n">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="L279" s="10" t="inlineStr">
         <is>
@@ -18715,7 +18715,7 @@
         </is>
       </c>
       <c r="K280" s="7" t="n">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="L280" s="7" t="inlineStr">
         <is>
@@ -18778,7 +18778,7 @@
         </is>
       </c>
       <c r="K281" s="10" t="n">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="L281" s="10" t="inlineStr">
         <is>
@@ -18841,7 +18841,7 @@
         </is>
       </c>
       <c r="K282" s="7" t="n">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="L282" s="7" t="inlineStr">
         <is>
@@ -18904,7 +18904,7 @@
         </is>
       </c>
       <c r="K283" s="10" t="n">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="L283" s="10" t="inlineStr">
         <is>
@@ -18967,7 +18967,7 @@
         </is>
       </c>
       <c r="K284" s="7" t="n">
-        <v>53</v>
+        <v>35</v>
       </c>
       <c r="L284" s="7" t="inlineStr">
         <is>
@@ -19030,7 +19030,7 @@
         </is>
       </c>
       <c r="K285" s="10" t="n">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="L285" s="10" t="inlineStr">
         <is>
@@ -19093,7 +19093,7 @@
         </is>
       </c>
       <c r="K286" s="7" t="n">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="L286" s="7" t="inlineStr">
         <is>
@@ -19156,7 +19156,7 @@
         </is>
       </c>
       <c r="K287" s="10" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="L287" s="10" t="inlineStr">
         <is>
@@ -19219,7 +19219,7 @@
         </is>
       </c>
       <c r="K288" s="7" t="n">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="L288" s="7" t="inlineStr">
         <is>
@@ -19282,7 +19282,7 @@
         </is>
       </c>
       <c r="K289" s="10" t="n">
-        <v>58</v>
+        <v>46</v>
       </c>
       <c r="L289" s="10" t="inlineStr">
         <is>
@@ -19345,7 +19345,7 @@
         </is>
       </c>
       <c r="K290" s="7" t="n">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="L290" s="7" t="inlineStr">
         <is>
@@ -19408,7 +19408,7 @@
         </is>
       </c>
       <c r="K291" s="10" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L291" s="10" t="inlineStr">
         <is>
@@ -19471,7 +19471,7 @@
         </is>
       </c>
       <c r="K292" s="7" t="n">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="L292" s="7" t="inlineStr">
         <is>
@@ -19534,7 +19534,7 @@
         </is>
       </c>
       <c r="K293" s="10" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="L293" s="10" t="inlineStr">
         <is>
@@ -19597,7 +19597,7 @@
         </is>
       </c>
       <c r="K294" s="7" t="n">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="L294" s="7" t="inlineStr">
         <is>
@@ -19660,7 +19660,7 @@
         </is>
       </c>
       <c r="K295" s="10" t="n">
-        <v>57</v>
+        <v>28</v>
       </c>
       <c r="L295" s="10" t="inlineStr">
         <is>
@@ -19723,7 +19723,7 @@
         </is>
       </c>
       <c r="K296" s="7" t="n">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="L296" s="7" t="inlineStr">
         <is>
@@ -19786,7 +19786,7 @@
         </is>
       </c>
       <c r="K297" s="10" t="n">
-        <v>33</v>
+        <v>15</v>
       </c>
       <c r="L297" s="10" t="inlineStr">
         <is>
@@ -19849,7 +19849,7 @@
         </is>
       </c>
       <c r="K298" s="7" t="n">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="L298" s="7" t="inlineStr">
         <is>
@@ -19912,7 +19912,7 @@
         </is>
       </c>
       <c r="K299" s="10" t="n">
-        <v>17</v>
+        <v>52</v>
       </c>
       <c r="L299" s="10" t="inlineStr">
         <is>
@@ -19975,7 +19975,7 @@
         </is>
       </c>
       <c r="K300" s="7" t="n">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="L300" s="7" t="inlineStr">
         <is>
@@ -20038,7 +20038,7 @@
         </is>
       </c>
       <c r="K301" s="10" t="n">
-        <v>29</v>
+        <v>50</v>
       </c>
       <c r="L301" s="10" t="inlineStr">
         <is>
@@ -20101,7 +20101,7 @@
         </is>
       </c>
       <c r="K302" s="7" t="n">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="L302" s="7" t="inlineStr">
         <is>
@@ -20164,7 +20164,7 @@
         </is>
       </c>
       <c r="K303" s="10" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="L303" s="10" t="inlineStr">
         <is>
@@ -20227,7 +20227,7 @@
         </is>
       </c>
       <c r="K304" s="7" t="n">
-        <v>16</v>
+        <v>41</v>
       </c>
       <c r="L304" s="7" t="inlineStr">
         <is>
@@ -20290,7 +20290,7 @@
         </is>
       </c>
       <c r="K305" s="10" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="L305" s="10" t="inlineStr">
         <is>
@@ -20353,7 +20353,7 @@
         </is>
       </c>
       <c r="K306" s="7" t="n">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="L306" s="7" t="inlineStr">
         <is>
@@ -20416,7 +20416,7 @@
         </is>
       </c>
       <c r="K307" s="10" t="n">
-        <v>44</v>
+        <v>19</v>
       </c>
       <c r="L307" s="10" t="inlineStr">
         <is>
@@ -20479,7 +20479,7 @@
         </is>
       </c>
       <c r="K308" s="7" t="n">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="L308" s="7" t="inlineStr">
         <is>
@@ -20542,7 +20542,7 @@
         </is>
       </c>
       <c r="K309" s="10" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="L309" s="10" t="inlineStr">
         <is>
@@ -20605,7 +20605,7 @@
         </is>
       </c>
       <c r="K310" s="7" t="n">
-        <v>55</v>
+        <v>32</v>
       </c>
       <c r="L310" s="7" t="inlineStr">
         <is>
@@ -20668,7 +20668,7 @@
         </is>
       </c>
       <c r="K311" s="10" t="n">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="L311" s="10" t="inlineStr">
         <is>

</xml_diff>